<commit_message>
fix(rewrite): preserve integer rounding and validated save recovery
</commit_message>
<xml_diff>
--- a/space-battleship/tests/excel/core_rules.xlsx
+++ b/space-battleship/tests/excel/core_rules.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -691,7 +691,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>N01-series</t>
+          <t>N01-int-floor</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -714,7 +714,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>N01-linear</t>
+          <t>N01-int-ceil</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -737,7 +737,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>N01-div-zero</t>
+          <t>N01-series</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -760,7 +760,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>N01-overflow</t>
+          <t>N01-linear</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -775,6 +775,52 @@
         <v>0.01666666666666667</v>
       </c>
       <c r="E15" t="inlineStr">
+        <is>
+          <t>amount_relative</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>N01-div-zero</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>core_rules</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>17</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.01666666666666667</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>amount_relative</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>N01-overflow</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>core_rules</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>17</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.01666666666666667</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>amount_relative</t>
         </is>
@@ -791,7 +837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1211,28 +1257,28 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>N01-series</t>
+          <t>N01-int-floor</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>sum_geometric</t>
+          <t>floor</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>113</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>113</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -1242,28 +1288,28 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>N01-linear</t>
+          <t>N01-int-ceil</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>sum_geometric</t>
+          <t>ceil</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2e500</t>
+          <t>201</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2e504</t>
+          <t>201</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -1273,33 +1319,28 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>N01-div-zero</t>
+          <t>N01-series</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>div</t>
+          <t>sum_geometric</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>AmountDivisionByZero</t>
+        <v>4</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>30</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -1309,36 +1350,103 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>N01-linear</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>sum_geometric</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2e500</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>10000</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2e504</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>1e-12</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>N01-div-zero</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>div</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>AmountDivisionByZero</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>1e-12</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>N01-overflow</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>mul</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>1e9000000000000000</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" t="inlineStr">
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="inlineStr">
         <is>
           <t>AmountRangeExceeded</t>
         </is>
       </c>
-      <c r="I15" t="n">
+      <c r="I17" t="n">
         <v>1e-12</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(config): enforce player equipment and resource cost required fields
</commit_message>
<xml_diff>
--- a/space-battleship/tests/excel/core_rules.xlsx
+++ b/space-battleship/tests/excel/core_rules.xlsx
@@ -1671,7 +1671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2017,6 +2017,42 @@
         <v>0.1</v>
       </c>
       <c r="O5" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>laser</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>fixture player</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" t="n">
+        <v>71</v>
+      </c>
+      <c r="J6" t="n">
+        <v>7</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O6" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(rewrite): migrate native combat amounts and retain cross-wave execution
</commit_message>
<xml_diff>
--- a/space-battleship/tests/excel/core_rules.xlsx
+++ b/space-battleship/tests/excel/core_rules.xlsx
@@ -9,12 +9,14 @@
   <sheets>
     <sheet name="case" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="amount_case" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="res" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="enemy_weapon_base" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="equipment" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="mon" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="monGroup" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="level" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="kernel_case" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="wave_case" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="res" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="enemy_weapon_base" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="equipment" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="mon" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="monGroup" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="level" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -420,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -824,6 +826,380 @@
         <is>
           <t>amount_relative</t>
         </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>C01-before</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>core_rules</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>17</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>native_exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>C01-after</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>core_rules</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>17</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>native_exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>C12-cannon</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>core_rules</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>17</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>native_exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>C07-missile</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>core_rules</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>17</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>native_exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>C08-beam</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>core_rules</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>17</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>native_exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>N01-native-large</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>core_rules</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>17</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>native_exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>W01</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>core_rules</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>17</v>
+      </c>
+      <c r="D24" t="n">
+        <v>4</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>native_wave</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>length</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>monGroup</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>atkRatio</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>lifeRatio</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>resRatio</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>jewelRatio</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>planetExpRatio</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>entryAtkRatio</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>entryLifeRatio</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>rewardReferenceGroups</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>9301</v>
+      </c>
+      <c r="B4" t="n">
+        <v>100</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>{9201|0.5}</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1461,30 +1837,230 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:V9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>case_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>damage</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>enemy_hp</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>enemy_shield</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>shield_type</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>resistance</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>interval</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>initial_delay</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>charge</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>maximum</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ramp</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>speed</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>duration</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>expected_hp</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>expected_shield</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>history_start</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>expected_attacks</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>enemy_x</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>enemy_y</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>player_x</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>player_y</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>independent</t>
+          <t>stage1 independent fixture</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>independent</t>
+          <t>stage1 independent fixture</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>stage1 independent fixture</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>stage1 independent fixture</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>stage1 independent fixture</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>stage1 independent fixture</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>stage1 independent fixture</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>stage1 independent fixture</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>stage1 independent fixture</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>stage1 independent fixture</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>stage1 independent fixture</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>stage1 independent fixture</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>stage1 independent fixture</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>stage1 independent fixture</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>stage1 independent fixture</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>stage1 independent fixture</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>stage1 independent fixture</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>stage1 independent fixture</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>stage1 independent fixture</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>stage1 independent fixture</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>stage1 independent fixture</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>stage1 independent fixture</t>
         </is>
       </c>
     </row>
@@ -1499,15 +2075,609 @@
           <t>literal</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>71</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>test_iron</t>
-        </is>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>C01-before</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H4" t="n">
+        <v>10</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>C01-after</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H5" t="n">
+        <v>10</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>960</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>C12-cannon</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H6" t="n">
+        <v>10</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" t="n">
+        <v>1000</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>960</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S6" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>C07-missile</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H7" t="n">
+        <v>10</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="N7" t="n">
+        <v>2</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>900</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>C08-beam</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="N8" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>900</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S8" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>N01-native-large</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1e500</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>1e501</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H9" t="n">
+        <v>10</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" t="n">
+        <v>1000</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>9e500</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>9007199254740993</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>9007199254740994</t>
+        </is>
+      </c>
+      <c r="S9" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" t="n">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1521,80 +2691,130 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>case_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>dmg</t>
+          <t>player_hp</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>cd</t>
+          <t>player_damage</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>dmgtype</t>
+          <t>player_interval</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>para1</t>
+          <t>enemy_hp</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>para2</t>
+          <t>enemy_damage</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>para3</t>
+          <t>enemy_interval</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>enemy_speed</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>distance</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>resource</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>drop_amount</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>travel_seconds</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>independent</t>
+          <t>stage1 independent fixture</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>independent</t>
+          <t>stage1 independent fixture</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>independent</t>
+          <t>stage1 independent fixture</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>independent</t>
+          <t>stage1 independent fixture</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>independent</t>
+          <t>stage1 independent fixture</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>independent</t>
+          <t>stage1 independent fixture</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>independent</t>
+          <t>stage1 independent fixture</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>stage1 independent fixture</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>stage1 independent fixture</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>stage1 independent fixture</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>stage1 independent fixture</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>stage1 independent fixture</t>
         </is>
       </c>
     </row>
@@ -1634,30 +2854,80 @@
           <t>literal</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>laser</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+          <t>W01</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="H4" t="n">
+        <v>50</v>
+      </c>
+      <c r="I4" t="n">
+        <v>100</v>
+      </c>
+      <c r="J4" t="n">
+        <v>71</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
         <v>3</v>
-      </c>
-      <c r="C4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" t="n">
-        <v>100</v>
-      </c>
-      <c r="F4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1671,93 +2941,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>name</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>des</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>level</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>dmgtype</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>dmg</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>dmgMulti</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>cd</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>res_1</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>cost_1</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>costMulti_1</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>res_2</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>cost_2</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>costMulti_2</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>para1</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>para2</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>para3</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>para4</t>
         </is>
       </c>
     </row>
@@ -1772,86 +2967,6 @@
           <t>independent</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1864,196 +2979,15 @@
           <t>literal</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>armour</t>
-        </is>
+      <c r="A4" t="n">
+        <v>71</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>fixture</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" t="n">
-        <v>2</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>71</v>
-      </c>
-      <c r="J4" t="n">
-        <v>7</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="O4" t="n">
-        <v>30</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>laser_mon</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>fixture enemy</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G5" t="n">
-        <v>2</v>
-      </c>
-      <c r="I5" t="n">
-        <v>71</v>
-      </c>
-      <c r="J5" t="n">
-        <v>7</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="O5" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>laser</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>fixture player</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" t="n">
-        <v>3</v>
-      </c>
-      <c r="G6" t="n">
-        <v>2</v>
-      </c>
-      <c r="I6" t="n">
-        <v>71</v>
-      </c>
-      <c r="J6" t="n">
-        <v>7</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="O6" t="n">
-        <v>100</v>
+          <t>test_iron</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2067,7 +3001,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2078,87 +3012,32 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>des</t>
+          <t>dmg</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>equipment</t>
+          <t>cd</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>dmgMultiple</t>
+          <t>dmgtype</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>para1</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>armourType</t>
+          <t>para2</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>res</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>size</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>shield</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>shieldType</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>shieldRecovery</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>shieldDelay</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>reactiveReduction</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>archetype_id</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>intelTrait</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>intelName</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>intelVisualRef</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>intelMechanics</t>
+          <t>para3</t>
         </is>
       </c>
     </row>
@@ -2198,61 +3077,6 @@
           <t>independent</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>independent</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2290,104 +3114,30 @@
           <t>literal</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>9101</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>fixture</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>{laser_mon|1}</t>
-        </is>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>laser</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>9</v>
+        <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>{71,2,1}</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>2</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2401,13 +3151,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>name</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -2417,12 +3167,77 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>mon</t>
+          <t>level</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>combatTier</t>
+          <t>dmgtype</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>dmg</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>dmgMulti</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>cd</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>res_1</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>cost_1</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>costMulti_1</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>res_2</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>cost_2</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>costMulti_2</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>para1</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>para2</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>para3</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>para4</t>
         </is>
       </c>
     </row>
@@ -2447,6 +3262,76 @@
           <t>independent</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2469,20 +3354,186 @@
           <t>literal</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>9201</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>armour</t>
+        </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
           <t>fixture</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>{null,null,null,9101,null,null,null,null,null,null}</t>
-        </is>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>71</v>
+      </c>
+      <c r="J4" t="n">
+        <v>7</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O4" t="n">
+        <v>30</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>laser_mon</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>fixture enemy</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" t="n">
+        <v>71</v>
+      </c>
+      <c r="J5" t="n">
+        <v>7</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O5" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>laser</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>fixture player</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" t="n">
+        <v>71</v>
+      </c>
+      <c r="J6" t="n">
+        <v>7</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O6" t="n">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -2496,7 +3547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2507,52 +3558,87 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>length</t>
+          <t>des</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>monGroup</t>
+          <t>equipment</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>atkRatio</t>
+          <t>dmgMultiple</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>lifeRatio</t>
+          <t>health</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>resRatio</t>
+          <t>armourType</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>jewelRatio</t>
+          <t>res</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>planetExpRatio</t>
+          <t>size</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>entryAtkRatio</t>
+          <t>shield</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>entryLifeRatio</t>
+          <t>shieldType</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>rewardReferenceGroups</t>
+          <t>shieldRecovery</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>shieldDelay</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>reactiveReduction</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>archetype_id</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>intelTrait</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>intelName</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>intelVisualRef</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>intelMechanics</t>
         </is>
       </c>
     </row>
@@ -2612,6 +3698,41 @@
           <t>independent</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2669,33 +3790,179 @@
           <t>literal</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>9301</v>
-      </c>
-      <c r="B4" t="n">
-        <v>100</v>
+        <v>9101</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>{9201|0.5}</t>
+          <t>{laser_mon|1}</t>
         </is>
       </c>
       <c r="D4" t="n">
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>{71,2,1}</t>
+        </is>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>des</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>mon</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>combatTier</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>independent</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>9201</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>{null,null,null,9101,null,null,null,null,null,null}</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Complete stage 2 native session, paid attributes and runtime verification
</commit_message>
<xml_diff>
--- a/space-battleship/tests/excel/core_rules.xlsx
+++ b/space-battleship/tests/excel/core_rules.xlsx
@@ -25,11 +25,15 @@
     <sheet name="journey_case" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="income_case" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="ratio_case" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="ship" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="config" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="enhance_config" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="unlock" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="weapon_motion" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="equipment_evolution" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="loadout_case" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="defence_case" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="geometry_case" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="ship" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="config" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="enhance_config" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="unlock" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="weapon_motion" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -435,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1411,6 +1415,144 @@
         <v>0.001</v>
       </c>
       <c r="E42" t="inlineStr">
+        <is>
+          <t>session_exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>L01-level2</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>core_rules</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>17</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>session_exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>L02-evolution20</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>core_rules</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>17</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>session_exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>M01-loss-authority</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>core_rules</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>17</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>session_exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>M02-large-loss</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>core_rules</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>17</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>session_exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>G01-empty15</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>core_rules</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>17</v>
+      </c>
+      <c r="D47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>session_exact</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>G02-full15</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>core_rules</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>17</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" t="inlineStr">
         <is>
           <t>session_exact</t>
         </is>
@@ -4512,43 +4654,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>des</t>
+          <t>interval</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>para_1</t>
+          <t>first_stat_multiplier</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>para_2</t>
+          <t>later_stat_multiplier</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>para_3</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>para_5</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>para_6</t>
+          <t>defence_growth</t>
         </is>
       </c>
     </row>
@@ -4578,21 +4710,6 @@
           <t>runtime contract</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>runtime contract</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>runtime contract</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>runtime contract</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4620,47 +4737,24 @@
           <t>literal</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>fixture_ship</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>independent fixture</t>
-        </is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>20</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>1.6</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="E4" t="n">
-        <v>50</v>
-      </c>
-      <c r="G4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H4" t="n">
-        <v>999</v>
+        <v>0.2</v>
       </c>
     </row>
   </sheetData>
@@ -5298,23 +5392,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>case_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>des</t>
+          <t>paid_level</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>para_1</t>
+          <t>expected_armour</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>expected_damage</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>expected_shield</t>
         </is>
       </c>
     </row>
@@ -5334,6 +5438,16 @@
           <t>runtime contract</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5351,21 +5465,64 @@
           <t>literal</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>startEquip</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>independent fixture</t>
-        </is>
+          <t>L01-level2</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>armour,laser</t>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>L02-evolution20</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1536</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>152</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>768</t>
         </is>
       </c>
     </row>
@@ -5380,28 +5537,53 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>case_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>base_a</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>base_b</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>des</t>
+          <t>loss_a</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>loss_b</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>expected_remaining</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>expected_loss_a</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>expected_loss_b</t>
         </is>
       </c>
     </row>
@@ -5426,6 +5608,31 @@
           <t>runtime contract</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5448,44 +5655,123 @@
           <t>literal</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>counter_log_base</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>10</v>
+          <t>M01-loss-authority</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>fixture</t>
+          <t>300</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>shared log base</t>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>280</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>bonus_round_scale</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>100</v>
+          <t>M02-large-loss</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1e500</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>fixture</t>
+          <t>3e500</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>shared precision</t>
+          <t>2e499</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>6e499</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>4e499</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2.8e500</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>3e499</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>9e499</t>
         </is>
       </c>
     </row>
@@ -5500,43 +5786,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>case_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>type</t>
+          <t>slots</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>target</t>
+          <t>target_slot</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>expected_x</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>mode</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>desc</t>
+          <t>expected_y</t>
         </is>
       </c>
     </row>
@@ -5566,16 +5842,6 @@
           <t>runtime contract</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>runtime contract</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>runtime contract</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5603,155 +5869,47 @@
           <t>literal</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>literal</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>armour</t>
+          <t>G01-empty15</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>equipment</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>armour</t>
-        </is>
+          <t>{9101,null,null,null,null,null,null,null,null,null,null,null,null,null,9101}</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>14</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>cleared</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>fixture</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>fixture</t>
-        </is>
+        <v>80</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>laser</t>
+          <t>G02-full15</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>equipment</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>laser</t>
-        </is>
+          <t>{9101,9101,9101,9101,9101,9101,9101,9101,9101,9101,9101,9101,9101,9101,9101}</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>10</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>cleared</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>fixture</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>fixture</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>fixture_ship</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>ship</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>fixture_ship</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>cleared</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>fixture</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>fixture</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>feature/jewels</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>feature</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>jewels</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>reached</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>fixture</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>fixture</t>
-        </is>
+      <c r="E5" t="n">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -5760,6 +5918,635 @@
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>des</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>para_1</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>para_2</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>para_3</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>para_5</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>para_6</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>fixture_ship</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>independent fixture</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>des</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>para_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>startEquip</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>independent fixture</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>armour,laser</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>des</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>counter_log_base</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>shared log base</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>bonus_round_scale</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>100</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>shared precision</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>level</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>mode</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>desc</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>runtime contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>literal</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>armour</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>equipment</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>armour</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>cleared</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>laser</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>equipment</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>laser</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>cleared</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>fixture_ship</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ship</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>fixture_ship</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>cleared</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>feature/jewels</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>feature</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>jewels</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>reached</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6730,7 +7517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:R7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7099,6 +7886,9 @@
       <c r="E6" t="n">
         <v>3</v>
       </c>
+      <c r="F6" t="n">
+        <v>0.2</v>
+      </c>
       <c r="G6" t="n">
         <v>2</v>
       </c>
@@ -7113,6 +7903,51 @@
       </c>
       <c r="O6" t="n">
         <v>100</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>shield</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>fixture</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>71</v>
+      </c>
+      <c r="J7" t="n">
+        <v>7</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O7" t="n">
+        <v>15</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>